<commit_message>
feat(parsing): prendre la première colonne par défaut + fichiers d'exemple
- ne considère la 1re ligne comme en-tête que si elle nomme une colonne
  ('Nom', 'Président'...) ; sinon toutes les lignes sont des données, pour
  qu'une simple liste ne perde jamais son premier nom
- décodage CSV explicite en UTF-8 (accents : René, Valéry... préservés)
- fichiers d'exemple (xlsx avec en-tête + csv brut) : présidents et figures
  politiques des IVe et Ve Républiques (58 noms)
</commit_message>
<xml_diff>
--- a/participants-exemple.xlsx
+++ b/participants-exemple.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A59"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -406,107 +406,297 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Yuki Tanaka</v>
+        <v>Vincent Auriol</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Hiroshi Sato</v>
+        <v>René Coty</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Aiko Yamamoto</v>
+        <v>Charles de Gaulle</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Kenji Nakamura</v>
+        <v>Georges Pompidou</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Sakura Ito</v>
+        <v>Valéry Giscard d’Estaing</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Ren Watanabe</v>
+        <v>François Mitterrand</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Mei Kobayashi</v>
+        <v>Jacques Chirac</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Sora Suzuki</v>
+        <v>Nicolas Sarkozy</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Haruto Takahashi</v>
+        <v>François Hollande</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Emi Kato</v>
+        <v>Emmanuel Macron</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Robin Straub</v>
+        <v>Pierre Mendès France</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Marie Dupont</v>
+        <v>Guy Mollet</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Lucas Bernard</v>
+        <v>Antoine Pinay</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Chloé Martin</v>
+        <v>Edgar Faure</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Thomas Petit</v>
+        <v>Robert Schuman</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Léa Moreau</v>
+        <v>Georges Bidault</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Antoine Girard</v>
+        <v>Henri Queuille</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Camille Laurent</v>
+        <v>René Pleven</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Julien Roux</v>
+        <v>Félix Gouin</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Manon Simon</v>
+        <v>Paul Ramadier</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Maurice Bourgès-Maunoury</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Félix Gaillard</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Pierre Pflimlin</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Michel Debré</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Maurice Couve de Murville</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Jacques Chaban-Delmas</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Pierre Messmer</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Raymond Barre</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Pierre Mauroy</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Laurent Fabius</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Michel Rocard</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Édith Cresson</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Pierre Bérégovoy</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Édouard Balladur</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Alain Juppé</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Lionel Jospin</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Jean-Pierre Raffarin</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Dominique de Villepin</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>François Fillon</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Manuel Valls</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Bernard Cazeneuve</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Édouard Philippe</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Jean Castex</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Élisabeth Borne</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Gabriel Attal</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Simone Veil</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Georges Marchais</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Jean-Marie Le Pen</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Marine Le Pen</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Jean-Luc Mélenchon</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Ségolène Royal</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Martine Aubry</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>François Bayrou</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Philippe Séguin</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Charles Pasqua</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Jack Lang</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Robert Badinter</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Michel Barnier</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A59"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>